<commit_message>
chore: run 2026-02-27 20:54 — histórico, dashboard e Excel atualizados
</commit_message>
<xml_diff>
--- a/logs/Consolidado_27_02_2026.xlsx
+++ b/logs/Consolidado_27_02_2026.xlsx
@@ -602,10 +602,10 @@
         <v>151</v>
       </c>
       <c r="C2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E2" t="n">
         <v>4</v>
@@ -659,10 +659,10 @@
         <v>72</v>
       </c>
       <c r="C5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E5" t="n">
         <v>3</v>
@@ -5851,40 +5851,40 @@
       </c>
     </row>
     <row r="129">
-      <c r="A129" s="3" t="inlineStr">
-        <is>
-          <t>27/02/2026</t>
-        </is>
-      </c>
-      <c r="B129" s="3" t="inlineStr">
+      <c r="A129" s="7" t="inlineStr">
+        <is>
+          <t>27/02/2026</t>
+        </is>
+      </c>
+      <c r="B129" s="7" t="inlineStr">
         <is>
           <t>Avène</t>
         </is>
       </c>
-      <c r="C129" s="3" t="inlineStr">
+      <c r="C129" s="7" t="inlineStr">
         <is>
           <t>Sun Care Ultra Fluid Mat-Perfect SPF50+
 Protetor Solar Fluido Rosto Mat Sensível Cor
 50 ml</t>
         </is>
       </c>
-      <c r="D129" s="3" t="inlineStr">
+      <c r="D129" s="7" t="inlineStr">
         <is>
           <t>https://wells.pt/sun-care-ultra-fluid-mat-perfect-spf50-7536016.html</t>
         </is>
       </c>
-      <c r="E129" s="3" t="inlineStr"/>
-      <c r="F129" s="4" t="inlineStr">
-        <is>
-          <t>In Stock</t>
-        </is>
-      </c>
-      <c r="G129" s="3" t="inlineStr">
+      <c r="E129" s="7" t="inlineStr"/>
+      <c r="F129" s="8" t="inlineStr">
+        <is>
+          <t>Out of Stock</t>
+        </is>
+      </c>
+      <c r="G129" s="7" t="inlineStr">
         <is>
           <t>7536016</t>
         </is>
       </c>
-      <c r="H129" s="3" t="inlineStr">
+      <c r="H129" s="7" t="inlineStr">
         <is>
           <t>50%</t>
         </is>
@@ -11852,7 +11852,7 @@
       </c>
       <c r="G43" s="3" t="inlineStr">
         <is>
-          <t>8544713</t>
+          <t>8544715</t>
         </is>
       </c>
       <c r="H43" s="3" t="inlineStr">
@@ -14505,40 +14505,40 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="inlineStr">
-        <is>
-          <t>27/02/2026</t>
-        </is>
-      </c>
-      <c r="B6" s="7" t="inlineStr">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>27/02/2026</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>René Furterer</t>
         </is>
       </c>
-      <c r="C6" s="7" t="inlineStr">
+      <c r="C6" s="3" t="inlineStr">
         <is>
           <t>Absolue Kératine Renewal Care Serum
 Sérum Reparador Extremo Pontas Danificadas
 30 ml</t>
         </is>
       </c>
-      <c r="D6" s="7" t="inlineStr">
+      <c r="D6" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/absolue-keratine-renewal-care-serum-7447296.html</t>
         </is>
       </c>
-      <c r="E6" s="7" t="inlineStr"/>
-      <c r="F6" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G6" s="7" t="inlineStr">
+      <c r="E6" s="3" t="inlineStr"/>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
         <is>
           <t>7447296</t>
         </is>
       </c>
-      <c r="H6" s="7" t="inlineStr">
+      <c r="H6" s="3" t="inlineStr">
         <is>
           <t>30%</t>
         </is>
@@ -21544,7 +21544,7 @@
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t>8544713</t>
+          <t>8544715</t>
         </is>
       </c>
       <c r="F40" s="5" t="inlineStr">

</xml_diff>

<commit_message>
chore: run 2026-02-27 21:52 — histórico, dashboard e Excel atualizados
</commit_message>
<xml_diff>
--- a/logs/Consolidado_27_02_2026.xlsx
+++ b/logs/Consolidado_27_02_2026.xlsx
@@ -15544,7 +15544,7 @@
       </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>6633968</t>
+          <t>5522799</t>
         </is>
       </c>
       <c r="H31" s="5" t="inlineStr">
@@ -15587,12 +15587,12 @@
       </c>
       <c r="G32" s="5" t="inlineStr">
         <is>
-          <t>7610972</t>
+          <t>5522799</t>
         </is>
       </c>
       <c r="H32" s="5" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>20%</t>
         </is>
       </c>
     </row>
@@ -22418,7 +22418,7 @@
       </c>
       <c r="E63" s="3" t="inlineStr">
         <is>
-          <t>6633968</t>
+          <t>5522799</t>
         </is>
       </c>
       <c r="F63" s="3" t="inlineStr">
@@ -22456,12 +22456,12 @@
       </c>
       <c r="E64" s="3" t="inlineStr">
         <is>
-          <t>7610972</t>
+          <t>5522799</t>
         </is>
       </c>
       <c r="F64" s="3" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>20%</t>
         </is>
       </c>
       <c r="G64" s="3" t="inlineStr">

</xml_diff>